<commit_message>
feat: activate excel product import with auto category/brand creation, fix quill view transitions bug
</commit_message>
<xml_diff>
--- a/public/downloads/ornek-urun-sablonu.xlsx
+++ b/public/downloads/ornek-urun-sablonu.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Ürünler" sheetId="1" r:id="rId1"/>
+    <sheet name="Ürün Şablonu" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:BE2"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="19.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="23.83203125" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="21.83203125" customWidth="1"/>
+    <col min="14" max="14" width="17.83203125" customWidth="1"/>
+    <col min="15" max="15" width="17.83203125" customWidth="1"/>
+    <col min="16" max="16" width="15.83203125" customWidth="1"/>
+    <col min="17" max="17" width="15.83203125" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" customWidth="1"/>
+    <col min="19" max="19" width="16.83203125" customWidth="1"/>
+    <col min="20" max="20" width="16.83203125" customWidth="1"/>
+    <col min="21" max="21" width="16.83203125" customWidth="1"/>
+    <col min="22" max="22" width="16.83203125" customWidth="1"/>
+    <col min="23" max="23" width="16.83203125" customWidth="1"/>
+    <col min="24" max="24" width="15.83203125" customWidth="1"/>
+    <col min="25" max="25" width="16.83203125" customWidth="1"/>
+    <col min="26" max="26" width="24.83203125" customWidth="1"/>
+    <col min="27" max="27" width="17.83203125" customWidth="1"/>
+    <col min="28" max="28" width="20.83203125" customWidth="1"/>
+    <col min="29" max="29" width="17.83203125" customWidth="1"/>
+    <col min="30" max="30" width="20.83203125" customWidth="1"/>
+    <col min="31" max="31" width="17.83203125" customWidth="1"/>
+    <col min="32" max="32" width="20.83203125" customWidth="1"/>
+    <col min="33" max="33" width="17.83203125" customWidth="1"/>
+    <col min="34" max="34" width="20.83203125" customWidth="1"/>
+    <col min="35" max="35" width="17.83203125" customWidth="1"/>
+    <col min="36" max="36" width="20.83203125" customWidth="1"/>
+    <col min="37" max="37" width="19.83203125" customWidth="1"/>
+    <col min="38" max="38" width="20.83203125" customWidth="1"/>
+    <col min="39" max="39" width="21.83203125" customWidth="1"/>
+    <col min="40" max="40" width="19.83203125" customWidth="1"/>
+    <col min="41" max="41" width="20.83203125" customWidth="1"/>
+    <col min="42" max="42" width="21.83203125" customWidth="1"/>
+    <col min="43" max="43" width="19.83203125" customWidth="1"/>
+    <col min="44" max="44" width="20.83203125" customWidth="1"/>
+    <col min="45" max="45" width="21.83203125" customWidth="1"/>
+    <col min="46" max="46" width="19.83203125" customWidth="1"/>
+    <col min="47" max="47" width="20.83203125" customWidth="1"/>
+    <col min="48" max="48" width="21.83203125" customWidth="1"/>
+    <col min="49" max="49" width="19.83203125" customWidth="1"/>
+    <col min="50" max="50" width="20.83203125" customWidth="1"/>
+    <col min="51" max="51" width="21.83203125" customWidth="1"/>
+    <col min="52" max="52" width="24.83203125" customWidth="1"/>
+    <col min="53" max="53" width="28.83203125" customWidth="1"/>
+    <col min="54" max="54" width="24.83203125" customWidth="1"/>
+    <col min="55" max="55" width="28.83203125" customWidth="1"/>
+    <col min="56" max="56" width="24.83203125" customWidth="1"/>
+    <col min="57" max="57" width="28.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,10 +466,10 @@
         <v>URL (Slug)</v>
       </c>
       <c r="C1" t="str">
-        <v>Kategori ID</v>
+        <v>Kategori</v>
       </c>
       <c r="D1" t="str">
-        <v>Marka ID</v>
+        <v>Marka</v>
       </c>
       <c r="E1" t="str">
         <v>Satış Fiyatı</v>
@@ -444,44 +503,170 @@
       </c>
       <c r="O1" t="str">
         <v>Sağ Üst Rozet</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Satıcı Adı</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Etiketler</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Ana Görsel URL</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Görsel 1 URL</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Görsel 2 URL</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Görsel 3 URL</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Görsel 4 URL</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Görsel 5 URL</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Video URL</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>Satış Birimi</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Min. Sipariş Miktarı</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Özellik Adı 1</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>Özellik Değeri 1</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>Özellik Adı 2</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Özellik Değeri 2</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>Özellik Adı 3</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Özellik Değeri 3</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Özellik Adı 4</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>Özellik Değeri 4</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>Özellik Adı 5</v>
+      </c>
+      <c r="AJ1" t="str">
+        <v>Özellik Değeri 5</v>
+      </c>
+      <c r="AK1" t="str">
+        <v>Varyasyon Adı 1</v>
+      </c>
+      <c r="AL1" t="str">
+        <v>Varyasyon Stok 1</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>Varyasyon Fiyat 1</v>
+      </c>
+      <c r="AN1" t="str">
+        <v>Varyasyon Adı 2</v>
+      </c>
+      <c r="AO1" t="str">
+        <v>Varyasyon Stok 2</v>
+      </c>
+      <c r="AP1" t="str">
+        <v>Varyasyon Fiyat 2</v>
+      </c>
+      <c r="AQ1" t="str">
+        <v>Varyasyon Adı 3</v>
+      </c>
+      <c r="AR1" t="str">
+        <v>Varyasyon Stok 3</v>
+      </c>
+      <c r="AS1" t="str">
+        <v>Varyasyon Fiyat 3</v>
+      </c>
+      <c r="AT1" t="str">
+        <v>Varyasyon Adı 4</v>
+      </c>
+      <c r="AU1" t="str">
+        <v>Varyasyon Stok 4</v>
+      </c>
+      <c r="AV1" t="str">
+        <v>Varyasyon Fiyat 4</v>
+      </c>
+      <c r="AW1" t="str">
+        <v>Varyasyon Adı 5</v>
+      </c>
+      <c r="AX1" t="str">
+        <v>Varyasyon Stok 5</v>
+      </c>
+      <c r="AY1" t="str">
+        <v>Varyasyon Fiyat 5</v>
+      </c>
+      <c r="AZ1" t="str">
+        <v>Toptan Min. Miktar 1</v>
+      </c>
+      <c r="BA1" t="str">
+        <v>Toptan İndirim Oranı % 1</v>
+      </c>
+      <c r="BB1" t="str">
+        <v>Toptan Min. Miktar 2</v>
+      </c>
+      <c r="BC1" t="str">
+        <v>Toptan İndirim Oranı % 2</v>
+      </c>
+      <c r="BD1" t="str">
+        <v>Toptan Min. Miktar 3</v>
+      </c>
+      <c r="BE1" t="str">
+        <v>Toptan İndirim Oranı % 3</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Örnek Ürün</v>
+        <v>Akıllı Akustik Bluetooth Hoparlör</v>
       </c>
       <c r="B2" t="str">
-        <v>ornek-urun</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
+        <v>akilli-akustik-bluetooth-hoparlor</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Teknoloji</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Samsung</v>
       </c>
       <c r="E2">
-        <v>299.9</v>
+        <v>1899.9</v>
       </c>
       <c r="F2">
-        <v>399.9</v>
+        <v>2499.9</v>
       </c>
       <c r="G2" t="str">
-        <v>SKU-1001</v>
+        <v>SKU-HPR-100</v>
       </c>
       <c r="H2" t="str">
-        <v>123456789</v>
+        <v>8681234567890</v>
       </c>
       <c r="I2">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="J2" t="str">
         <v>aktif</v>
       </c>
       <c r="K2" t="str">
-        <v>Kısa bilgi...</v>
+        <v>Yüksek kaliteli ses performansı sunan akıllı bluetooth hoparlör.</v>
       </c>
       <c r="L2" t="str">
-        <v>&lt;p&gt;Detaylı HTML içeriği&lt;/p&gt;</v>
+        <v>&lt;p&gt;Samsung Akıllı Akustik Bluetooth Hoparlör ile evinizde konser salonu deneyimini yaşayın. 360 derece ses dağılımı, derin baslar ve net tiz sesler ile müzik keyfinizi zirveye taşıyın.&lt;/p&gt;</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -490,12 +675,138 @@
         <v>Yeni</v>
       </c>
       <c r="O2" t="str">
-        <v>Kampanya</v>
+        <v>Ücretsiz Kargo</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Samsung Türkiye</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>hoparlör,bluetooth,ses,teknoloji,samsung</v>
+      </c>
+      <c r="R2" t="str">
+        <v>https://images.unsplash.com/photo-1608043152269-423dbba4e7e1?q=80&amp;w=600&amp;auto=format&amp;fit=crop</v>
+      </c>
+      <c r="S2" t="str">
+        <v>https://images.unsplash.com/photo-1545454675-3531b543be5d?q=80&amp;w=600&amp;auto=format&amp;fit=crop</v>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v>https://www.youtube.com/watch?v=dQw4w9WgXcQ</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Adet</v>
+      </c>
+      <c r="Z2">
+        <v>1</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>Renk</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>Kömür Grisi</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>Bağlantı</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>Bluetooth 5.2</v>
+      </c>
+      <c r="AE2" t="str">
+        <v>Güç</v>
+      </c>
+      <c r="AF2" t="str">
+        <v>40W RMS</v>
+      </c>
+      <c r="AG2" t="str">
+        <v>Pil Ömrü</v>
+      </c>
+      <c r="AH2" t="str">
+        <v>12 Saate Kadar</v>
+      </c>
+      <c r="AI2" t="str">
+        <v>Suya Dayanıklılık</v>
+      </c>
+      <c r="AJ2" t="str">
+        <v>IPX7 Sertifikalı</v>
+      </c>
+      <c r="AK2" t="str">
+        <v>Gri - Standart</v>
+      </c>
+      <c r="AL2">
+        <v>50</v>
+      </c>
+      <c r="AM2">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="str">
+        <v>Siyah - Pro Kit</v>
+      </c>
+      <c r="AO2">
+        <v>40</v>
+      </c>
+      <c r="AP2">
+        <v>400</v>
+      </c>
+      <c r="AQ2" t="str">
+        <v>Beyaz - Special Edition</v>
+      </c>
+      <c r="AR2">
+        <v>30</v>
+      </c>
+      <c r="AS2">
+        <v>150</v>
+      </c>
+      <c r="AT2" t="str">
+        <v/>
+      </c>
+      <c r="AU2" t="str">
+        <v/>
+      </c>
+      <c r="AV2" t="str">
+        <v/>
+      </c>
+      <c r="AW2" t="str">
+        <v/>
+      </c>
+      <c r="AX2" t="str">
+        <v/>
+      </c>
+      <c r="AY2" t="str">
+        <v/>
+      </c>
+      <c r="AZ2">
+        <v>5</v>
+      </c>
+      <c r="BA2">
+        <v>10</v>
+      </c>
+      <c r="BB2">
+        <v>10</v>
+      </c>
+      <c r="BC2">
+        <v>15</v>
+      </c>
+      <c r="BD2">
+        <v>20</v>
+      </c>
+      <c r="BE2">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:BE2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>